<commit_message>
updated with all scenarios and step definitions
</commit_message>
<xml_diff>
--- a/src/main/resources/eureka.xlsx
+++ b/src/main/resources/eureka.xlsx
@@ -1,19 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{554006D2-5DDB-4520-91BB-F306C59A8602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\SeleniumWorkSpaceEclipse\edureka-automation-testing\src\main\resources\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76BAF4FE-31ED-4ACF-8CB9-72FBEC8E1B05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{B61975A8-7105-4470-A3D6-068E94FB6268}"/>
+    <workbookView xWindow="2370" yWindow="2265" windowWidth="17520" windowHeight="8655" activeTab="3" xr2:uid="{B61975A8-7105-4470-A3D6-068E94FB6268}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="AuthData" sheetId="2" r:id="rId2"/>
     <sheet name="BlogData" sheetId="3" r:id="rId3"/>
+    <sheet name="CommunityQuestions" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:M11"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -23,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t>email</t>
   </si>
@@ -71,6 +76,27 @@
   </si>
   <si>
     <t>Test Comment</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Tag</t>
+  </si>
+  <si>
+    <t>Selenium issue in POM while working with BDD</t>
+  </si>
+  <si>
+    <t>Selenium</t>
+  </si>
+  <si>
+    <t>This problems arise when the POM is used along with BDD</t>
+  </si>
+  <si>
+    <t>java</t>
   </si>
 </sst>
 </file>
@@ -448,7 +474,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{111011FA-C08A-4F01-B9B7-9E860A471529}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -457,13 +483,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6343EBA-F3DC-423D-B377-70F5249FB146}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29" customWidth="1"/>
-    <col min="2" max="2" width="21.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -471,7 +497,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -490,17 +516,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33633261-1C6C-486C-BD2E-03EF2FD4779E}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.44140625" customWidth="1"/>
-    <col min="2" max="2" width="15.33203125" customWidth="1"/>
-    <col min="3" max="3" width="16.88671875" customWidth="1"/>
-    <col min="4" max="4" width="15.6640625" customWidth="1"/>
+    <col min="1" max="1" width="15.42578125" customWidth="1"/>
+    <col min="2" max="2" width="15.28515625" customWidth="1"/>
+    <col min="3" max="3" width="16.85546875" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="16.21875" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
@@ -520,7 +546,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
@@ -538,6 +564,50 @@
       </c>
       <c r="F2" s="3" t="s">
         <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA711BC9-A1D5-4B65-951C-7144E9AA05F5}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="44" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated with postjob module
</commit_message>
<xml_diff>
--- a/src/main/resources/eureka.xlsx
+++ b/src/main/resources/eureka.xlsx
@@ -1,34 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\SeleniumWorkSpaceEclipse\edureka-automation-testing\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sathy\eclipse-workspace\seleniumTraining\Edureka_Automation_Testing\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76BAF4FE-31ED-4ACF-8CB9-72FBEC8E1B05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{914033AE-5102-4E58-B8B5-98C8D5EC12A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2370" yWindow="2265" windowWidth="17520" windowHeight="8655" activeTab="3" xr2:uid="{B61975A8-7105-4470-A3D6-068E94FB6268}"/>
+    <workbookView xWindow="1740" yWindow="1740" windowWidth="8330" windowHeight="7270" xr2:uid="{B61975A8-7105-4470-A3D6-068E94FB6268}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="SearchData" sheetId="1" r:id="rId1"/>
     <sheet name="AuthData" sheetId="2" r:id="rId2"/>
     <sheet name="BlogData" sheetId="3" r:id="rId3"/>
     <sheet name="CommunityQuestions" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="37">
   <si>
     <t>email</t>
   </si>
@@ -97,6 +106,48 @@
   </si>
   <si>
     <t>java</t>
+  </si>
+  <si>
+    <t>validKeyword</t>
+  </si>
+  <si>
+    <t>invalidKeyword</t>
+  </si>
+  <si>
+    <t>specialKeyword</t>
+  </si>
+  <si>
+    <t>popularKeyword</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>validMobile</t>
+  </si>
+  <si>
+    <t>invalidMobile</t>
+  </si>
+  <si>
+    <t>python</t>
+  </si>
+  <si>
+    <t>xyz123invalid</t>
+  </si>
+  <si>
+    <t>@@@###</t>
+  </si>
+  <si>
+    <t>devops</t>
+  </si>
+  <si>
+    <t>DevOps</t>
+  </si>
+  <si>
+    <t>9876543210</t>
+  </si>
+  <si>
+    <t>9876543210123</t>
   </si>
 </sst>
 </file>
@@ -149,13 +200,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -473,9 +527,56 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{111011FA-C08A-4F01-B9B7-9E860A471529}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -483,13 +584,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6343EBA-F3DC-423D-B377-70F5249FB146}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="29" customWidth="1"/>
-    <col min="2" max="2" width="21.28515625" customWidth="1"/>
+    <col min="2" max="2" width="21.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -497,7 +598,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -516,17 +617,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33633261-1C6C-486C-BD2E-03EF2FD4779E}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.42578125" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" customWidth="1"/>
-    <col min="3" max="3" width="16.85546875" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="15.453125" customWidth="1"/>
+    <col min="2" max="2" width="15.26953125" customWidth="1"/>
+    <col min="3" max="3" width="16.81640625" customWidth="1"/>
+    <col min="4" max="4" width="15.7265625" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="16.28515625" customWidth="1"/>
+    <col min="6" max="6" width="16.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
@@ -546,7 +647,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
@@ -574,15 +675,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA711BC9-A1D5-4B65-951C-7144E9AA05F5}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="44" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="53.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>16</v>
       </c>
@@ -596,7 +697,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>19</v>
       </c>

</xml_diff>

<commit_message>
Updated with Comments, Extent reports - All course module
</commit_message>
<xml_diff>
--- a/src/main/resources/eureka.xlsx
+++ b/src/main/resources/eureka.xlsx
@@ -3,22 +3,19 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sathy\eclipse-workspace\seleniumTraining\Edureka_Automation_Testing\src\main\resources\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{914033AE-5102-4E58-B8B5-98C8D5EC12A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{BEB5E15B-877E-41F6-B40B-0D3647A53148}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1740" yWindow="1740" windowWidth="8330" windowHeight="7270" xr2:uid="{B61975A8-7105-4470-A3D6-068E94FB6268}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{B61975A8-7105-4470-A3D6-068E94FB6268}"/>
   </bookViews>
   <sheets>
     <sheet name="SearchData" sheetId="1" r:id="rId1"/>
-    <sheet name="AuthData" sheetId="2" r:id="rId2"/>
-    <sheet name="BlogData" sheetId="3" r:id="rId3"/>
-    <sheet name="CommunityQuestions" sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="5" r:id="rId2"/>
+    <sheet name="AuthData" sheetId="2" r:id="rId3"/>
+    <sheet name="BlogData" sheetId="3" r:id="rId4"/>
+    <sheet name="CommunityQuestions" sheetId="4" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1:O7"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="41">
   <si>
     <t>email</t>
   </si>
@@ -148,6 +145,18 @@
   </si>
   <si>
     <t>9876543210123</t>
+  </si>
+  <si>
+    <t>course</t>
+  </si>
+  <si>
+    <t>phone</t>
+  </si>
+  <si>
+    <t>Tableau Certification Training Course</t>
+  </si>
+  <si>
+    <t>test@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -200,7 +209,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -210,6 +219,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -231,9 +243,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -271,7 +283,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -377,7 +389,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -519,7 +531,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -528,9 +540,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{111011FA-C08A-4F01-B9B7-9E860A471529}">
   <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>23</v>
       </c>
@@ -553,7 +565,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>30</v>
       </c>
@@ -582,15 +594,50 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED223D28-1E44-4A86-B887-6E90F2564441}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" display="mailto:test@gmail.com" xr:uid="{810F4732-7EDC-4A63-8B64-80CD2707A46C}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6343EBA-F3DC-423D-B377-70F5249FB146}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29" customWidth="1"/>
-    <col min="2" max="2" width="21.26953125" customWidth="1"/>
+    <col min="2" max="2" width="21.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -598,7 +645,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -614,20 +661,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33633261-1C6C-486C-BD2E-03EF2FD4779E}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.453125" customWidth="1"/>
-    <col min="2" max="2" width="15.26953125" customWidth="1"/>
-    <col min="3" max="3" width="16.81640625" customWidth="1"/>
-    <col min="4" max="4" width="15.7265625" customWidth="1"/>
+    <col min="1" max="1" width="15.44140625" customWidth="1"/>
+    <col min="2" max="2" width="15.21875" customWidth="1"/>
+    <col min="3" max="3" width="16.77734375" customWidth="1"/>
+    <col min="4" max="4" width="15.77734375" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="16.26953125" customWidth="1"/>
+    <col min="6" max="6" width="16.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
@@ -647,7 +694,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="58" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
@@ -672,18 +719,18 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA711BC9-A1D5-4B65-951C-7144E9AA05F5}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="44" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="53.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>16</v>
       </c>
@@ -697,7 +744,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>19</v>
       </c>

</xml_diff>